<commit_message>
Use explicit sheet keys and document local builder outputs
</commit_message>
<xml_diff>
--- a/templates/practice-calculators.xlsx
+++ b/templates/practice-calculators.xlsx
@@ -2447,19 +2447,19 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B14" location="'Allocation'!B2" display="Allocation" xr:uid="{01B06C28-D813-4AFE-9DE2-C1AF086E62EC}"/>
-    <hyperlink ref="B15" location="'Contractor'!B2" display="Contractor" xr:uid="{26929B88-952C-47F0-A628-80EB1DA813E1}"/>
-    <hyperlink ref="B16" location="'Vendor finance'!B2" display="Vendor finance" xr:uid="{13C3A877-F2F1-494A-8586-6BB5A49473BD}"/>
-    <hyperlink ref="B17" location="'Mixed loan'!B2" display="Mixed loan" xr:uid="{433DC501-5F5E-44D8-A494-F72D74D84A89}"/>
-    <hyperlink ref="B18" location="'Rental'!B2" display="Rental" xr:uid="{E293B8E4-BC4E-4994-8140-D374783193E5}"/>
-    <hyperlink ref="B19" location="'Packaging'!B2" display="Packaging" xr:uid="{A6C3AC5A-F71E-49AF-9066-7E68037F955D}"/>
-    <hyperlink ref="B20" location="'Amortisation'!B2" display="Amortisation" xr:uid="{84BA9047-00F5-4826-A2A1-DFD3FEAFB981}"/>
-    <hyperlink ref="B21" location="'Timeline'!B2" display="Timeline" xr:uid="{97389819-55A6-48FA-B587-054CCB43DB9B}"/>
-    <hyperlink ref="B22" location="'Deed register'!B2" display="Deed register" xr:uid="{A6E95E1D-B4C8-4E77-BA3F-4C072AD9F042}"/>
-    <hyperlink ref="B23" location="'Carry forward'!B2" display="Carry forward" xr:uid="{1ADC7228-3ECF-43A4-A989-9839CFBD3849}"/>
-    <hyperlink ref="B24" location="'Loan offers'!B2" display="Loan offers" xr:uid="{2E50D3D4-51A5-42F0-9550-892ACF981698}"/>
-    <hyperlink ref="B25" location="'Break even'!B2" display="Break even" xr:uid="{2F67F8D1-0870-4EAF-BCEF-C8A7BE94EDC6}"/>
-    <hyperlink ref="B26" location="'Working capital'!B2" display="Working capital" xr:uid="{EC01953E-2072-4332-B62F-83303F084890}"/>
+    <hyperlink ref="B14" location="'Allocation'!B2" display="Allocation" xr:uid="{526EB053-7368-4B1D-804C-5AC0A59111CB}"/>
+    <hyperlink ref="B15" location="'Contractor'!B2" display="Contractor" xr:uid="{1DD1B0E3-F9F8-4A19-9AA3-5F4FF0634792}"/>
+    <hyperlink ref="B16" location="'Vendor finance'!B2" display="Vendor finance" xr:uid="{4C4F4937-460D-4808-894C-8D90BB37C539}"/>
+    <hyperlink ref="B17" location="'Mixed loan'!B2" display="Mixed loan" xr:uid="{8EA8D4A3-FE92-48B0-8CAD-E77D1164CCD8}"/>
+    <hyperlink ref="B18" location="'Rental'!B2" display="Rental" xr:uid="{FE18D7E9-B992-4B6E-BD48-5352EA8B1FC4}"/>
+    <hyperlink ref="B19" location="'Packaging'!B2" display="Packaging" xr:uid="{6FFA111F-33C7-47CD-8E82-B8096D6A2755}"/>
+    <hyperlink ref="B20" location="'Amortisation'!B2" display="Amortisation" xr:uid="{930F7DFE-8BC4-44B7-9D0D-613DBD2C1133}"/>
+    <hyperlink ref="B21" location="'Timeline'!B2" display="Timeline" xr:uid="{6451D052-12CE-4E02-A18C-96DF686069B1}"/>
+    <hyperlink ref="B22" location="'Deed register'!B2" display="Deed register" xr:uid="{31E9C6C7-B7D5-45CE-802C-B39E49710641}"/>
+    <hyperlink ref="B23" location="'Carry forward'!B2" display="Carry forward" xr:uid="{BF9B77A5-EF03-4AFB-A886-C75BA6A9872B}"/>
+    <hyperlink ref="B24" location="'Loan offers'!B2" display="Loan offers" xr:uid="{6CA4D250-AA72-48CF-AF76-508A5386B749}"/>
+    <hyperlink ref="B25" location="'Break even'!B2" display="Break even" xr:uid="{228F9791-9B19-4670-8D72-99D73A6766AB}"/>
+    <hyperlink ref="B26" location="'Working capital'!B2" display="Working capital" xr:uid="{DDF00B45-A037-4C19-AD1C-96EE7026349A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3294,7 +3294,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{FB80ECE1-DCB3-4916-BA2A-48C8FBF80C10}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{E7CC174D-5619-42D2-95D3-7CE9214E8082}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4191,7 +4191,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{61D85308-E366-4946-9DFC-698A2E423E2C}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{C295FEB7-C3F5-4140-BFA4-9981897B035B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5212,7 +5212,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{DD88E0FE-2866-44CA-B83D-CDE0603253C7}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{F6FE35AA-12F8-4D1A-A439-80098C1C7597}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6028,7 +6028,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{91F67580-8DA7-4486-A67C-864E4929CECE}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{89F51E8A-E5D2-4FB2-A1F0-274147ECE855}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6856,7 +6856,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{9D9882F3-1EC4-4442-BCD8-7890A71D6FA8}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{E8317834-0090-41DD-BE79-AAF90DCB45F3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8893,7 +8893,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{DEA2AAF1-1AC1-443A-8301-DC2C5B188695}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{26FED839-9EBB-4177-8342-9A7DA594E2EE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9697,7 +9697,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{94494CFC-04C8-44FA-B16E-508D0560BFC6}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{716879D0-46AD-4261-9B30-9B6D7101EAE6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10783,7 +10783,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{CF6B938E-7803-4AAB-8E37-C3FA75CB7D34}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{3FCBB31E-D4BB-4915-A163-7F6640B2BD35}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17514,7 +17514,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{1EA02D4E-AF08-43D1-9E42-8A71100F9FAF}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{88FE2CF3-2C71-46F7-94B6-7DE85DA1C7B2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -18540,7 +18540,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{04B0E626-7BAD-4C7F-A727-515598FFBAE7}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{00D7A09A-9FA3-48A0-A18E-64119D833DF6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19378,7 +19378,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{67001625-5E66-44B5-8DC6-FABCFC8C1772}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{02667EF4-DE96-48B3-B05D-7DEA862470BA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21097,7 +21097,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{FB4EACA8-AE24-49A5-B076-4C0EA38AD8DC}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{C0410A12-EB17-4AF2-B7AC-CB62D279EC06}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23729,7 +23729,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{F39A1807-12A6-43CF-A171-FF9B230D613F}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{B7CA81BF-77E3-4DEA-8BC8-1EF19F90D248}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Bound amortisation remainders and extend native precision checks
</commit_message>
<xml_diff>
--- a/templates/practice-calculators.xlsx
+++ b/templates/practice-calculators.xlsx
@@ -3271,27 +3271,27 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B14" location="'Allocation'!B2" display="Allocation" xr:uid="{2EF71553-D471-4F41-AF38-62F57C07A55C}"/>
-    <hyperlink ref="B15" location="'Contractor'!B2" display="Contractor" xr:uid="{6F8DE2A7-AC8B-465B-AE2B-8BBF98B607D5}"/>
-    <hyperlink ref="B16" location="'Vendor finance'!B2" display="Vendor finance" xr:uid="{6A0BA88C-E225-451B-AC0D-3BB970266768}"/>
-    <hyperlink ref="B17" location="'Mixed loan'!B2" display="Mixed loan" xr:uid="{D46B7D4E-B6E8-4F1E-AE44-F4E8B8F2F8BF}"/>
-    <hyperlink ref="B18" location="'Rental'!B2" display="Rental" xr:uid="{DFD15FD4-5CEA-46DD-8F6A-CA3B4369F372}"/>
-    <hyperlink ref="B19" location="'Packaging'!B2" display="Packaging" xr:uid="{B9AC3170-8317-4345-B75C-28791265FFBA}"/>
-    <hyperlink ref="B20" location="'Amortisation'!B2" display="Amortisation" xr:uid="{391BC94B-F265-4B88-B084-A7C5BFD294A5}"/>
-    <hyperlink ref="B21" location="'Timeline'!B2" display="Timeline" xr:uid="{4AFA6E42-ECC6-40F6-A0D7-D04C423E49CC}"/>
-    <hyperlink ref="B22" location="'Deed register'!B2" display="Deed register" xr:uid="{E75E61E6-4D65-4AD3-AF21-642A508D1EA9}"/>
-    <hyperlink ref="B23" location="'Carry forward'!B2" display="Carry forward" xr:uid="{1B6512B1-F27D-418F-99FC-A87872119833}"/>
-    <hyperlink ref="B24" location="'Loan offers'!B2" display="Loan offers" xr:uid="{644E8B4B-3095-48BF-8348-CDFCC8824801}"/>
-    <hyperlink ref="B25" location="'Break even'!B2" display="Break even" xr:uid="{44D47EF2-70B1-4C11-AB36-3263FB8AD7AC}"/>
-    <hyperlink ref="B26" location="'Working capital'!B2" display="Working capital" xr:uid="{465D6536-64B3-4004-A2CC-D2B6F60C87BF}"/>
-    <hyperlink ref="B27" location="'Construction WIP'!B2" display="Construction WIP" xr:uid="{093785F6-66C0-4D52-81E4-2558AD89E347}"/>
-    <hyperlink ref="B28" location="'KPI awards'!B2" display="KPI awards" xr:uid="{2469F274-CC42-457C-8A46-6494F8C9B759}"/>
-    <hyperlink ref="B29" location="'Asset disposal'!B2" display="Asset disposal" xr:uid="{E11CB855-0BFA-4B75-8BAD-6AA13D3D8D63}"/>
-    <hyperlink ref="B30" location="'Exit pay'!B2" display="Exit pay" xr:uid="{50779DF5-BCF5-4A61-A3E0-00B087B984E5}"/>
-    <hyperlink ref="B31" location="'Tax cash'!B2" display="Tax cash" xr:uid="{5E2E01C6-DEE2-4AB1-83AA-CAAA91A42A04}"/>
-    <hyperlink ref="B32" location="'Investment'!B2" display="Investment" xr:uid="{5175DFA9-6A4A-4B65-B3FF-D50CA260E20A}"/>
-    <hyperlink ref="B33" location="'Action register'!B2" display="Action register" xr:uid="{B65AA20E-90F4-4E47-85BC-88B98DAAEE28}"/>
-    <hyperlink ref="B34" location="'Benefit totals'!B2" display="Benefit totals" xr:uid="{CFA2C6E6-02B2-4618-869D-5E0605E72F06}"/>
+    <hyperlink ref="B14" location="'Allocation'!B2" display="Allocation" xr:uid="{3FE609D7-8553-4F2E-99A3-3C8EC37128C3}"/>
+    <hyperlink ref="B15" location="'Contractor'!B2" display="Contractor" xr:uid="{CAF55CEC-B555-4E71-B29E-FC927A85E1AA}"/>
+    <hyperlink ref="B16" location="'Vendor finance'!B2" display="Vendor finance" xr:uid="{CA4E9E5A-F3A5-4DA4-932E-0345D02C00A0}"/>
+    <hyperlink ref="B17" location="'Mixed loan'!B2" display="Mixed loan" xr:uid="{A070C0F5-15BC-4E98-AE60-375A4901B89C}"/>
+    <hyperlink ref="B18" location="'Rental'!B2" display="Rental" xr:uid="{9D0358A1-5211-4892-8D40-E8DFDB960539}"/>
+    <hyperlink ref="B19" location="'Packaging'!B2" display="Packaging" xr:uid="{BB774975-61C5-4D18-9E5E-1217A293AA3B}"/>
+    <hyperlink ref="B20" location="'Amortisation'!B2" display="Amortisation" xr:uid="{CF8A7C6C-65DB-4BA5-86C9-2E8086138FBA}"/>
+    <hyperlink ref="B21" location="'Timeline'!B2" display="Timeline" xr:uid="{A1530804-50A1-4D01-B0CB-85240E4B8644}"/>
+    <hyperlink ref="B22" location="'Deed register'!B2" display="Deed register" xr:uid="{5F809364-0440-49CC-82A4-6615E1F1792D}"/>
+    <hyperlink ref="B23" location="'Carry forward'!B2" display="Carry forward" xr:uid="{6A55D44C-5BA7-4958-BD24-A805D485AB45}"/>
+    <hyperlink ref="B24" location="'Loan offers'!B2" display="Loan offers" xr:uid="{0D13FAFC-8891-48CF-A1C8-8E4175F3EFA3}"/>
+    <hyperlink ref="B25" location="'Break even'!B2" display="Break even" xr:uid="{6748D6C6-8451-4E72-97E0-68A10B3C4040}"/>
+    <hyperlink ref="B26" location="'Working capital'!B2" display="Working capital" xr:uid="{E420C37A-7CA0-4A7E-832B-AE567A6DC078}"/>
+    <hyperlink ref="B27" location="'Construction WIP'!B2" display="Construction WIP" xr:uid="{3F837D17-0EE6-460E-8427-E45BC9ACE8C0}"/>
+    <hyperlink ref="B28" location="'KPI awards'!B2" display="KPI awards" xr:uid="{86603040-F2FF-40E0-BA6D-EE683E42F5A0}"/>
+    <hyperlink ref="B29" location="'Asset disposal'!B2" display="Asset disposal" xr:uid="{BC424518-E52A-4689-A70E-83C87981E4AD}"/>
+    <hyperlink ref="B30" location="'Exit pay'!B2" display="Exit pay" xr:uid="{D26C7F8F-6153-4613-883B-6B6E6F836279}"/>
+    <hyperlink ref="B31" location="'Tax cash'!B2" display="Tax cash" xr:uid="{12E3FE37-8EA9-48FF-862E-5858C6C81C6E}"/>
+    <hyperlink ref="B32" location="'Investment'!B2" display="Investment" xr:uid="{C8E998DC-18F6-48D9-81C5-12859AFE206B}"/>
+    <hyperlink ref="B33" location="'Action register'!B2" display="Action register" xr:uid="{E457A552-3DBD-4F78-B64E-8D0C99421EE9}"/>
+    <hyperlink ref="B34" location="'Benefit totals'!B2" display="Benefit totals" xr:uid="{719A1D23-747D-45C4-A685-2EC41AD9D209}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4126,7 +4126,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{705D1093-C3CA-4C4C-B789-C0F0663CB5DB}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{E23E7871-715F-4B92-A1CD-D1F51F5D8A04}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5023,7 +5023,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{177A40AC-D077-4321-96E9-435829724A13}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{80F438BC-5718-47C2-B4B9-FDBF7568D5C1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6044,7 +6044,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{A91AF09A-3BB4-40C3-A8A7-C8F9DE9C2A43}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{E6CFC8B1-9D51-4631-8766-3728D7B1DF94}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6860,7 +6860,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{295BE0D1-CB66-4B31-9850-8DAAEFDA0087}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{44334D9B-B72D-4041-AEAE-7B0D40F9DA90}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7688,7 +7688,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{7CC737BC-F55C-43F0-B8C5-2165EEE8A498}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{E07D696D-3470-4B35-9D01-2497BC7D03EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8940,7 +8940,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{86718517-B77F-4701-8FB5-AE051CCADB6A}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{1E73D2C2-20CB-4D41-88B0-602DBE2B241C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10057,7 +10057,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{312225F4-28A3-4BFD-91A6-B70189F356DE}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{5890494A-282B-4909-8B5C-0EE2E76735C8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11188,7 +11188,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{986F3461-B219-4C6C-BCD9-9A80B9FFAB9C}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{DDAE00C7-7FCE-4461-A2A3-9B4C03F421C3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12508,7 +12508,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{54C6F7CC-34DF-4F34-B70D-09C85CA1927C}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{0FB92FCC-0DCB-49E8-93BD-0271002F2879}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13458,7 +13458,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{398CA2A8-97A3-4BD2-A31E-3776FD8E629B}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{90410787-1E5B-4FB5-80A2-C69F8F0EA28E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15495,7 +15495,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{13E5FAC8-D49C-424D-BA88-A4395512A09A}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{A483909F-9F74-4853-9868-8D12D497BA53}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16919,7 +16919,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{332C27E3-9AF4-4BA7-BC9A-3B2AFA7660CC}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{E3CA1F1E-F71B-452B-BE63-DB979921BEE6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17931,7 +17931,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{C41D42CD-2DCB-4D13-B456-30A7BBB85169}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{4D45D462-E8C4-4421-ABE1-D30A78B84F01}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19034,7 +19034,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{8740FFA7-48E4-4CA3-A4B9-E8F7CE9A2F35}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{726839F3-87D4-4519-BE47-CCF532F93829}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19838,7 +19838,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{927AA248-4399-4DDB-BB3A-D85F5D69AD63}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{71DF8DF0-CEDA-457B-9F18-7DEDB2683EBF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -20924,7 +20924,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{FDB29811-2E8A-432E-AD20-A2613CEED334}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{0F328A3D-9ADF-4056-ADBC-95AFD83071A8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -28417,7 +28417,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{2F9CFDFB-F6D1-476D-8919-8A4955ED00AD}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{205B15FB-724B-42E3-86C8-CDE279121AE0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -29443,7 +29443,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{151D73A9-2DCE-4176-A396-EDA0D5EFE14C}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{4AD993B1-62E9-4E96-8739-5219E089DFD7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30370,7 +30370,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{465CD0EA-A18F-4FED-AD25-6A765CF042A9}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{7968F7B8-8A1D-4D80-A4F4-DF3A8DA18A94}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30637,47 +30637,47 @@
         <v>0</v>
       </c>
       <c r="H9" s="11">
-        <f t="shared" ref="H9:H19" si="0">IF($U9="Ready",IF(OR(H$8&lt;$F9,H$8&gt;$F9+$E9,AND($G9&gt;0,H$8&gt;$G9)),0,IF(AND($G9&gt;0,H$8=$G9),$C9-$D9-0,MIN($C9-$D9-0,($C9-$D9)/$E9*IF(H$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="H9:H19" si="0">IF($U9="Ready",IF(OR(H$8&lt;$F9,H$8&gt;$F9+$E9,AND($G9&gt;0,H$8&gt;$G9)),0,IF(AND($G9&gt;0,H$8=$G9),MAX(0,$C9-$D9-0),MIN(MAX(0,$C9-$D9-0),($C9-$D9)/$E9*IF(H$8=$F9,$V9,1)))),NA())</f>
         <v>1000</v>
       </c>
       <c r="I9" s="11">
-        <f t="shared" ref="I9:I19" si="1">IF($U9="Ready",IF(OR(I$8&lt;$F9,I$8&gt;$F9+$E9,AND($G9&gt;0,I$8&gt;$G9)),0,IF(AND($G9&gt;0,I$8=$G9),$C9-$D9-SUM(H9:H9),MIN($C9-$D9-SUM(H9:H9),($C9-$D9)/$E9*IF(I$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="I9:I19" si="1">IF($U9="Ready",IF(OR(I$8&lt;$F9,I$8&gt;$F9+$E9,AND($G9&gt;0,I$8&gt;$G9)),0,IF(AND($G9&gt;0,I$8=$G9),MAX(0,$C9-$D9-SUM(H9:H9)),MIN(MAX(0,$C9-$D9-SUM(H9:H9)),($C9-$D9)/$E9*IF(I$8=$F9,$V9,1)))),NA())</f>
         <v>1000</v>
       </c>
       <c r="J9" s="11">
-        <f t="shared" ref="J9:J19" si="2">IF($U9="Ready",IF(OR(J$8&lt;$F9,J$8&gt;$F9+$E9,AND($G9&gt;0,J$8&gt;$G9)),0,IF(AND($G9&gt;0,J$8=$G9),$C9-$D9-SUM(H9:I9),MIN($C9-$D9-SUM(H9:I9),($C9-$D9)/$E9*IF(J$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="J9:J19" si="2">IF($U9="Ready",IF(OR(J$8&lt;$F9,J$8&gt;$F9+$E9,AND($G9&gt;0,J$8&gt;$G9)),0,IF(AND($G9&gt;0,J$8=$G9),MAX(0,$C9-$D9-SUM(H9:I9)),MIN(MAX(0,$C9-$D9-SUM(H9:I9)),($C9-$D9)/$E9*IF(J$8=$F9,$V9,1)))),NA())</f>
         <v>1000</v>
       </c>
       <c r="K9" s="11">
-        <f t="shared" ref="K9:K19" si="3">IF($U9="Ready",IF(OR(K$8&lt;$F9,K$8&gt;$F9+$E9,AND($G9&gt;0,K$8&gt;$G9)),0,IF(AND($G9&gt;0,K$8=$G9),$C9-$D9-SUM(H9:J9),MIN($C9-$D9-SUM(H9:J9),($C9-$D9)/$E9*IF(K$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="K9:K19" si="3">IF($U9="Ready",IF(OR(K$8&lt;$F9,K$8&gt;$F9+$E9,AND($G9&gt;0,K$8&gt;$G9)),0,IF(AND($G9&gt;0,K$8=$G9),MAX(0,$C9-$D9-SUM(H9:J9)),MIN(MAX(0,$C9-$D9-SUM(H9:J9)),($C9-$D9)/$E9*IF(K$8=$F9,$V9,1)))),NA())</f>
         <v>1000</v>
       </c>
       <c r="L9" s="11">
-        <f t="shared" ref="L9:L19" si="4">IF($U9="Ready",IF(OR(L$8&lt;$F9,L$8&gt;$F9+$E9,AND($G9&gt;0,L$8&gt;$G9)),0,IF(AND($G9&gt;0,L$8=$G9),$C9-$D9-SUM(H9:K9),MIN($C9-$D9-SUM(H9:K9),($C9-$D9)/$E9*IF(L$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="L9:L19" si="4">IF($U9="Ready",IF(OR(L$8&lt;$F9,L$8&gt;$F9+$E9,AND($G9&gt;0,L$8&gt;$G9)),0,IF(AND($G9&gt;0,L$8=$G9),MAX(0,$C9-$D9-SUM(H9:K9)),MIN(MAX(0,$C9-$D9-SUM(H9:K9)),($C9-$D9)/$E9*IF(L$8=$F9,$V9,1)))),NA())</f>
         <v>1000</v>
       </c>
       <c r="M9" s="11">
-        <f t="shared" ref="M9:M19" si="5">IF($U9="Ready",IF(OR(M$8&lt;$F9,M$8&gt;$F9+$E9,AND($G9&gt;0,M$8&gt;$G9)),0,IF(AND($G9&gt;0,M$8=$G9),$C9-$D9-SUM(H9:L9),MIN($C9-$D9-SUM(H9:L9),($C9-$D9)/$E9*IF(M$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="M9:M19" si="5">IF($U9="Ready",IF(OR(M$8&lt;$F9,M$8&gt;$F9+$E9,AND($G9&gt;0,M$8&gt;$G9)),0,IF(AND($G9&gt;0,M$8=$G9),MAX(0,$C9-$D9-SUM(H9:L9)),MIN(MAX(0,$C9-$D9-SUM(H9:L9)),($C9-$D9)/$E9*IF(M$8=$F9,$V9,1)))),NA())</f>
         <v>0</v>
       </c>
       <c r="N9" s="11">
-        <f t="shared" ref="N9:N19" si="6">IF($U9="Ready",IF(OR(N$8&lt;$F9,N$8&gt;$F9+$E9,AND($G9&gt;0,N$8&gt;$G9)),0,IF(AND($G9&gt;0,N$8=$G9),$C9-$D9-SUM(H9:M9),MIN($C9-$D9-SUM(H9:M9),($C9-$D9)/$E9*IF(N$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="N9:N19" si="6">IF($U9="Ready",IF(OR(N$8&lt;$F9,N$8&gt;$F9+$E9,AND($G9&gt;0,N$8&gt;$G9)),0,IF(AND($G9&gt;0,N$8=$G9),MAX(0,$C9-$D9-SUM(H9:M9)),MIN(MAX(0,$C9-$D9-SUM(H9:M9)),($C9-$D9)/$E9*IF(N$8=$F9,$V9,1)))),NA())</f>
         <v>0</v>
       </c>
       <c r="O9" s="11">
-        <f t="shared" ref="O9:O19" si="7">IF($U9="Ready",IF(OR(O$8&lt;$F9,O$8&gt;$F9+$E9,AND($G9&gt;0,O$8&gt;$G9)),0,IF(AND($G9&gt;0,O$8=$G9),$C9-$D9-SUM(H9:N9),MIN($C9-$D9-SUM(H9:N9),($C9-$D9)/$E9*IF(O$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="O9:O19" si="7">IF($U9="Ready",IF(OR(O$8&lt;$F9,O$8&gt;$F9+$E9,AND($G9&gt;0,O$8&gt;$G9)),0,IF(AND($G9&gt;0,O$8=$G9),MAX(0,$C9-$D9-SUM(H9:N9)),MIN(MAX(0,$C9-$D9-SUM(H9:N9)),($C9-$D9)/$E9*IF(O$8=$F9,$V9,1)))),NA())</f>
         <v>0</v>
       </c>
       <c r="P9" s="11">
-        <f t="shared" ref="P9:P19" si="8">IF($U9="Ready",IF(OR(P$8&lt;$F9,P$8&gt;$F9+$E9,AND($G9&gt;0,P$8&gt;$G9)),0,IF(AND($G9&gt;0,P$8=$G9),$C9-$D9-SUM(H9:O9),MIN($C9-$D9-SUM(H9:O9),($C9-$D9)/$E9*IF(P$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="P9:P19" si="8">IF($U9="Ready",IF(OR(P$8&lt;$F9,P$8&gt;$F9+$E9,AND($G9&gt;0,P$8&gt;$G9)),0,IF(AND($G9&gt;0,P$8=$G9),MAX(0,$C9-$D9-SUM(H9:O9)),MIN(MAX(0,$C9-$D9-SUM(H9:O9)),($C9-$D9)/$E9*IF(P$8=$F9,$V9,1)))),NA())</f>
         <v>0</v>
       </c>
       <c r="Q9" s="11">
-        <f t="shared" ref="Q9:Q19" si="9">IF($U9="Ready",IF(OR(Q$8&lt;$F9,Q$8&gt;$F9+$E9,AND($G9&gt;0,Q$8&gt;$G9)),0,IF(AND($G9&gt;0,Q$8=$G9),$C9-$D9-SUM(H9:P9),MIN($C9-$D9-SUM(H9:P9),($C9-$D9)/$E9*IF(Q$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="Q9:Q19" si="9">IF($U9="Ready",IF(OR(Q$8&lt;$F9,Q$8&gt;$F9+$E9,AND($G9&gt;0,Q$8&gt;$G9)),0,IF(AND($G9&gt;0,Q$8=$G9),MAX(0,$C9-$D9-SUM(H9:P9)),MIN(MAX(0,$C9-$D9-SUM(H9:P9)),($C9-$D9)/$E9*IF(Q$8=$F9,$V9,1)))),NA())</f>
         <v>0</v>
       </c>
       <c r="R9" s="11">
-        <f t="shared" ref="R9:R19" si="10">IF($U9="Ready",IF(OR(R$8&lt;$F9,R$8&gt;$F9+$E9,AND($G9&gt;0,R$8&gt;$G9)),0,IF(AND($G9&gt;0,R$8=$G9),$C9-$D9-SUM(H9:Q9),MIN($C9-$D9-SUM(H9:Q9),($C9-$D9)/$E9*IF(R$8=$F9,$V9,1)))),NA())</f>
+        <f t="shared" ref="R9:R19" si="10">IF($U9="Ready",IF(OR(R$8&lt;$F9,R$8&gt;$F9+$E9,AND($G9&gt;0,R$8&gt;$G9)),0,IF(AND($G9&gt;0,R$8=$G9),MAX(0,$C9-$D9-SUM(H9:Q9)),MIN(MAX(0,$C9-$D9-SUM(H9:Q9)),($C9-$D9)/$E9*IF(R$8=$F9,$V9,1)))),NA())</f>
         <v>0</v>
       </c>
       <c r="S9" s="11">
@@ -30685,7 +30685,7 @@
         <v>5000</v>
       </c>
       <c r="T9" s="11">
-        <f t="shared" ref="T9:T19" si="12">C9-S9</f>
+        <f t="shared" ref="T9:T19" si="12">MAX(D9,C9-S9)</f>
         <v>0</v>
       </c>
       <c r="U9" s="15" t="str">
@@ -32160,7 +32160,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{35BCD4CA-9EAC-48BC-86B6-0E3851474FAE}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{9C26F549-9EEB-4AEB-802B-0CE7194A213E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -34792,7 +34792,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{F84ED4F2-2F4A-46AB-A09D-1183FA523869}"/>
+    <hyperlink ref="B1" location="'Read me'!B2" display="Contents" xr:uid="{FAD946A8-5E8E-4ACB-9F3B-BD75668A6D84}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>